<commit_message>
Dashboard V7 and scraper updates
</commit_message>
<xml_diff>
--- a/all_captured_1cr_tenders.xlsx
+++ b/all_captured_1cr_tenders.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>687.</t>
+          <t>736.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2003.</t>
+          <t>2017.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>910.</t>
+          <t>959.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>24.</t>
+          <t>31.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>165.</t>
+          <t>175.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2380.</t>
+          <t>2394.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5198.</t>
+          <t>5322.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>669.</t>
+          <t>679.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>752.</t>
+          <t>756.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1016,7 +1016,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>142.</t>
+          <t>164.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2237.</t>
+          <t>2354.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>372.</t>
+          <t>390.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5094.</t>
+          <t>5218.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>243.</t>
+          <t>250.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1306,7 +1306,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1656.</t>
+          <t>1786.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3848.</t>
+          <t>3976.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4070.</t>
+          <t>4197.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>4094.</t>
+          <t>4221.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5248.</t>
+          <t>5372.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2700.</t>
+          <t>2829.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1392.</t>
+          <t>1406.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">

</xml_diff>

<commit_message>
Updated tender keywords and filters
</commit_message>
<xml_diff>
--- a/all_captured_1cr_tenders.xlsx
+++ b/all_captured_1cr_tenders.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,7 +494,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>783.</t>
+          <t>1017.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1854.</t>
+          <t>1794.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2128.</t>
+          <t>1994.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Uttarakhand eTenders</t>
+          <t>Haryana eTenders</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -668,45 +668,45 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>312.</t>
+          <t>45.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>12-Jun-2026 04:15 PM</t>
+          <t>22-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>30-Jun-2026 12:30 PM</t>
+          <t>15-Jul-2026 05:00 PM</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>30-Jun-2026 01:00 PM</t>
+          <t>16-Jul-2026 09:00 AM</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[Construction of non-residential office building of Rural Works Department Division Rudraprayag in village Raitoli under district Rudraprayag.] [267/R.W.D/T.I-02/2026-27][2026_RES_96577_2]</t>
+          <t>[Construction of building of...] [2026C9E1FE7F 993F 4754 8589 4DC15137F937645BAR][2026_HRY_530778_1]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>RES - Chief Engineer||SE - Pauri||EE - Pauri</t>
+          <t>Haryana Government||Engineer-in-Chief PW(B and R) Department||SE Karnal||EE PD-2 Karnal</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2,91,40,100</t>
+          <t>9,55,97,065</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>29140100</v>
+        <v>95597065</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>https://uktenders.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=Sr16X%2F03zxO9kqVRVCdU%2FXg%3D%3D</t>
+          <t>https://etenders.hry.nic.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=S4di%2FBfHQPp6IR%2FBTk5jLxQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -718,7 +718,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Himachal eTenders</t>
+          <t>Uttarakhand eTenders</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -726,45 +726,45 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>806.</t>
+          <t>8.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>12-Jun-2026 11:00 AM</t>
+          <t>22-Jun-2026 04:15 PM</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>22-Jun-2026 05:00 PM</t>
+          <t>06-Jul-2026 03:00 PM</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>23-Jun-2026 11:00 AM</t>
+          <t>06-Jul-2026 03:30 PM</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[Construction of RTO Office Building at Nahan, Distt. Sirmour (HP).] [Job No. 4][2026_SIDC_136318_1]</t>
+          <t>[Construction of Proposed Regional Office Building for Pollution Board at Dehradun.] [962/BRIDCUL/1077/26 Dated 19.06.2026][2026_BRID3_96886_1]</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>HP SIDC Limited</t>
+          <t>MD - BRIDCUL||General Manager (Civil/Project)||PM (Dehradun)||JE</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2,79,52,391</t>
+          <t>4,50,46,000</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>27952391</v>
+        <v>45046000</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://hptenders.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SaPZgiL2NlyjRgJ5H4WKunw%3D%3D</t>
+          <t>https://uktenders.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SYU8Olh4hsb5k%2FPoIJVb%2FAQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Haryana eTenders</t>
+          <t>Uttarakhand eTenders</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -784,45 +784,45 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2315.</t>
+          <t>333.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>01-May-2026 03:00 PM</t>
+          <t>12-Jun-2026 04:15 PM</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>25-Jun-2026 05:00 PM</t>
+          <t>30-Jun-2026 12:30 PM</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>26-Jun-2026 11:00 AM</t>
+          <t>30-Jun-2026 01:00 PM</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[Construction of building for the Center for Distance and Online Education at 1st floor of building of University Works Department at GJU SandT, Hisar] [20262EB9E91C DD60 44A8 8F26 855DAA2E38B61129GJU][2026_HRY_519090_1]</t>
+          <t>[Construction of non-residential office building of Rural Works Department Division Rudraprayag in village Raitoli under district Rudraprayag.] [267/R.W.D/T.I-02/2026-27][2026_RES_96577_2]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Haryana Government||GJUS and T Hisar</t>
+          <t>RES - Chief Engineer||SE - Pauri||EE - Pauri</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1,58,61,542</t>
+          <t>2,91,40,100</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>15861542</v>
+        <v>29140100</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>https://etenders.hry.nic.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=S7%2B3mMyKcPocPDYXPM0hGCw%3D%3D</t>
+          <t>https://uktenders.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=Sr16X%2F03zxO9kqVRVCdU%2FXg%3D%3D</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Punjab eProcurement</t>
+          <t>Haryana eTenders</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -842,45 +842,45 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>942.</t>
+          <t>2160.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15-Jun-2026 09:00 AM</t>
+          <t>01-May-2026 03:00 PM</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>29-Jun-2026 01:00 PM</t>
+          <t>25-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>30-Jun-2026 09:00 AM</t>
+          <t>26-Jun-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[Construction of Building and playground of Govt. Sen. Sec. School (Girls) main bazar, Bhargo Camp.] [MCJ/(B and R) 2026-27/09][2026_DLG_169930_63]</t>
+          <t>[Construction of building for the Center for Distance and Online Education at 1st floor of building of University Works Department at GJU SandT, Hisar] [20262EB9E91C DD60 44A8 8F26 855DAA2E38B61129GJU][2026_HRY_519090_1]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Department of Local Government||Director - Local Government||Municipal Corporation - Jalandhar||B and R</t>
+          <t>Haryana Government||GJUS and T Hisar</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1,10,00,000</t>
+          <t>1,58,61,542</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>11000000</v>
+        <v>15861542</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://eproc.punjab.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=So%2F7JtzasXBC3D2YwSvhRtw%3D%3D</t>
+          <t>https://etenders.hry.nic.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=S7%2B3mMyKcPocPDYXPM0hGCw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -892,7 +892,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rajasthan eProcurement</t>
+          <t>Punjab eProcurement</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -900,45 +900,45 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6162.</t>
+          <t>1004.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>14-May-2026 06:00 PM</t>
+          <t>15-Jun-2026 09:00 AM</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>23-Jun-2026 02:00 PM</t>
+          <t>29-Jun-2026 01:00 PM</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>25-Jun-2026 04:00 PM</t>
+          <t>30-Jun-2026 09:00 AM</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[Const. of Division /Sub-Division office building (Vig) and Protection at Jalore] [Nit01/2026-27][2026_JdVVN_558872_11]</t>
+          <t>[Construction of Building and playground of Govt. Sen. Sec. School (Girls) main bazar, Bhargo Camp.] [MCJ/(B and R) 2026-27/09][2026_DLG_169930_63]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Jodhpur VVNL - MD||CE (HQ)||SE(CIVIL)||TA to SE(CIVIL), JODHPUR</t>
+          <t>Department of Local Government||Director - Local Government||Municipal Corporation - Jalandhar||B and R</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1,00,00,000</t>
+          <t>1,10,00,000</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>10000000</v>
+        <v>11000000</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SNkhzU01BT2m0XCYhaGOUUQ%3D%3D</t>
+          <t>https://eproc.punjab.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=So%2F7JtzasXBC3D2YwSvhRtw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -950,53 +950,53 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Haryana eTenders</t>
+          <t>Rajasthan eProcurement</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1401.</t>
+          <t>5975.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>15-Jun-2026 05:00 PM</t>
+          <t>14-May-2026 06:00 PM</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>25-Jun-2026 05:00 PM</t>
+          <t>23-Jun-2026 02:00 PM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>26-Jun-2026 09:00 AM</t>
+          <t>25-Jun-2026 04:00 PM</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[Construction of Library in ...] [2026125F74B7 AD39 48A3 A12F 6DE8C0F8C500345ULB][2026_HRY_529347_1]</t>
+          <t>[Const. of Division /Sub-Division office building (Vig) and Protection at Jalore] [Nit01/2026-27][2026_JdVVN_558872_11]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Haryana Government||Urban Local Bodies||MC Barwala</t>
+          <t>Jodhpur VVNL - MD||CE (HQ)||SE(CIVIL)||TA to SE(CIVIL), JODHPUR</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3,19,84,321</t>
+          <t>1,00,00,000</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>31984321</v>
+        <v>10000000</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>https://etenders.hry.nic.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SA2Kjj28gTwLxF2UEZTLzsw%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SNkhzU01BT2m0XCYhaGOUUQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Central eProcure</t>
+          <t>Haryana eTenders</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1016,45 +1016,45 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1228.</t>
+          <t>1516.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>12-Jun-2026 04:00 PM</t>
+          <t>15-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>24-Jun-2026 11:00 AM</t>
+          <t>25-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>25-Jun-2026 11:30 AM</t>
+          <t>26-Jun-2026 09:00 AM</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[CONSTRUCTION OF QUARTER GUARD BUILDING AT BSF CAMPUS BOI, DISTT. KANGRA OF 185 BN BSF (NOW 24 BN BSF) UNDER SHQ BSF GSP] [10/HQSDGWC/Engg/BSF/NIT/CO W/2026-27][2026_BSF_912822_1]</t>
+          <t>[Construction of Library in ...] [2026125F74B7 AD39 48A3 A12F 6DE8C0F8C500345ULB][2026_HRY_529347_1]</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DG,BSF,MHA||Punjab Ftr(Jallundhar),BSF,MHA</t>
+          <t>Haryana Government||Urban Local Bodies||MC Barwala</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>3,18,03,649</t>
+          <t>3,19,84,321</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>31803649</v>
+        <v>31984321</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://eprocure.gov.in/eprocure/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=ST0y9WeppUHo6r4QjpFCucw%3D%3D</t>
+          <t>https://etenders.hry.nic.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SA2Kjj28gTwLxF2UEZTLzsw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Punjab eProcurement</t>
+          <t>Central eProcure</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1074,103 +1074,103 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1293.</t>
+          <t>1285.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>10-Jun-2026 05:00 PM</t>
+          <t>12-Jun-2026 04:00 PM</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>24-Jun-2026 05:00 PM</t>
+          <t>24-Jun-2026 11:00 AM</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>25-Jun-2026 11:00 AM</t>
+          <t>25-Jun-2026 11:30 AM</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[CONSTRUCTION OF COMMUNITY HALL NEAR CHURCH CIVIL LINE AT HOSHIARPUR (PUNJAB)] [11][2026_CEPW_169887_1]</t>
+          <t>[CONSTRUCTION OF QUARTER GUARD BUILDING AT BSF CAMPUS BOI, DISTT. KANGRA OF 185 BN BSF (NOW 24 BN BSF) UNDER SHQ BSF GSP] [10/HQSDGWC/Engg/BSF/NIT/CO W/2026-27][2026_BSF_912822_1]</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>CE-PWD(B and R)||Construction Circle-Hoshiarpur||Provincial Division-Hoshiarpur</t>
+          <t>DG,BSF,MHA||Punjab Ftr(Jallundhar),BSF,MHA</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1,67,51,919</t>
+          <t>3,18,03,649</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>16751919</v>
+        <v>31803649</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://eproc.punjab.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=S%2F%2Ft7YZXMaRvO80hFY4Uwmw%3D%3D</t>
+          <t>https://eprocure.gov.in/eprocure/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=ST0y9WeppUHo6r4QjpFCucw%3D%3D</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Captured Backup</t>
+          <t>Review Tender</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rajasthan eProcurement</t>
+          <t>Punjab eProcurement</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6082.</t>
+          <t>1230.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>21-May-2026 05:00 PM</t>
+          <t>10-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>23-Jun-2026 02:00 PM</t>
+          <t>24-Jun-2026 05:00 PM</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>25-Jun-2026 02:00 PM</t>
+          <t>25-Jun-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[Construction of Building and Boundary wall at 04 Nos 33 kv s/s at Bijariya Bawadi (under Tinwari S/D), Hanuman Sagar (under Chamu S/D), Hapasar (under Sekhala S/D), Sadul Nagar (under Chamu S/D) under Distt. Circle), Jodhpur] [NIT 01/26-27 JU][2026_JdVVN_561401_1]</t>
+          <t>[CONSTRUCTION OF COMMUNITY HALL NEAR CHURCH CIVIL LINE AT HOSHIARPUR (PUNJAB)] [11][2026_CEPW_169887_1]</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Jodhpur VVNL - MD||CE (HQ)||SE(CIVIL)||TA to SE(CIVIL), JODHPUR</t>
+          <t>CE-PWD(B and R)||Construction Circle-Hoshiarpur||Provincial Division-Hoshiarpur</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1,34,50,000</t>
+          <t>1,67,51,919</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>13450000</v>
+        <v>16751919</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SKOJOYsCWuD7th2nNI3TIng%3D%3D</t>
+          <t>https://eproc.punjab.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=S%2F%2Ft7YZXMaRvO80hFY4Uwmw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1186,49 +1186,49 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>5317.</t>
+          <t>5898.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>10-Jun-2026 04:50 PM</t>
+          <t>21-May-2026 05:00 PM</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>02-Jul-2026 06:00 PM</t>
+          <t>23-Jun-2026 02:00 PM</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>03-Jul-2026 11:00 AM</t>
+          <t>25-Jun-2026 02:00 PM</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Kota. (Civil, Electric, Sanitary, Joinery works)] [EE M and H Kota NIT No. 04/2026-27][2026_MEDIC_565771_1]</t>
+          <t>[Construction of Building and Boundary wall at 04 Nos 33 kv s/s at Bijariya Bawadi (under Tinwari S/D), Hanuman Sagar (under Chamu S/D), Hapasar (under Sekhala S/D), Sadul Nagar (under Chamu S/D) under Distt. Circle), Jodhpur] [NIT 01/26-27 JU][2026_JdVVN_561401_1]</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Medical and Health</t>
+          <t>Jodhpur VVNL - MD||CE (HQ)||SE(CIVIL)||TA to SE(CIVIL), JODHPUR</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>5,00,00,000</t>
+          <t>1,34,50,000</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>50000000</v>
+        <v>13450000</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SJlGBFf4g9fkxvXcsRC5fGA%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SKOJOYsCWuD7th2nNI3TIng%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1248,32 +1248,32 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5809.</t>
+          <t>5220.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>04-Jun-2026 05:05 PM</t>
+          <t>10-Jun-2026 04:50 PM</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>24-Jun-2026 06:00 PM</t>
+          <t>02-Jul-2026 06:00 PM</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>25-Jun-2026 11:00 AM</t>
+          <t>03-Jul-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jaipur-II. (Civil, Sanitary, Joinery works)] [NIT No.05/2026-27EEM and HDiv 2 Jaipur/][2026_MEDIC_564977_1]</t>
+          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Kota. (Civil, Electric, Sanitary, Joinery works)] [EE M and H Kota NIT No. 04/2026-27][2026_MEDIC_565771_1]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Medical and Health||Chief Engineer</t>
+          <t>Medical and Health</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SHZR5G1CZ1n2laFIQysmK4g%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SJlGBFf4g9fkxvXcsRC5fGA%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5836.</t>
+          <t>5656.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>04-Jun-2026 10:00 AM</t>
+          <t>04-Jun-2026 05:05 PM</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>23-Jun-2026 06:00 PM</t>
+          <t>24-Jun-2026 06:00 PM</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>24-Jun-2026 11:00 AM</t>
+          <t>25-Jun-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under Jurisdiction of NHM Division Sawai Madhopur (Civil, Sanitary, Joinery works)] [Nit No. 04/2026-27 Executive Engineer Medical and Health Sawai Madhopur][2026_MEDIC_564750_1]</t>
+          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jaipur-II. (Civil, Sanitary, Joinery works)] [NIT No.05/2026-27EEM and HDiv 2 Jaipur/][2026_MEDIC_564977_1]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=Sww%2B5SwrMryuSox7h9K39OQ%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SHZR5G1CZ1n2laFIQysmK4g%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1364,12 +1364,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5842.</t>
+          <t>5682.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>04-Jun-2026 09:00 AM</t>
+          <t>04-Jun-2026 10:00 AM</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jodhpur (Civil, Sanitary, Joinery works)] [Nit No. 09/2026-27 of EE M and Jodhpur][2026_MEDIC_564531_1]</t>
+          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under Jurisdiction of NHM Division Sawai Madhopur (Civil, Sanitary, Joinery works)] [Nit No. 04/2026-27 Executive Engineer Medical and Health Sawai Madhopur][2026_MEDIC_564750_1]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1402,7 +1402,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SS7B95%2BlKtxmHztYWSYQXkQ%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=Sww%2B5SwrMryuSox7h9K39OQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1422,27 +1422,27 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6191.</t>
+          <t>5688.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>08-May-2026 09:00 AM</t>
+          <t>04-Jun-2026 09:00 AM</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>02-Jul-2026 06:00 PM</t>
+          <t>23-Jun-2026 06:00 PM</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>03-Jul-2026 11:00 AM</t>
+          <t>24-Jun-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jaipur-I. (Civil, Sanitary, Joinery works)] [NIT 09 2026-27 divi jaipurI][2026_MEDIC_557384_1]</t>
+          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jodhpur (Civil, Sanitary, Joinery works)] [Nit No. 09/2026-27 of EE M and Jodhpur][2026_MEDIC_564531_1]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SqdkfmioPRgMN%2BuVcWZkXJw%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SS7B95%2BlKtxmHztYWSYQXkQ%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1480,27 +1480,27 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5679.</t>
+          <t>6003.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>08-Jun-2026 04:00 PM</t>
+          <t>08-May-2026 09:00 AM</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>29-Jun-2026 06:00 PM</t>
+          <t>02-Jul-2026 06:00 PM</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>30-Jun-2026 01:00 PM</t>
+          <t>03-Jul-2026 11:00 AM</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>[Rate contract for General Repair and Maintenance Work at Various Hospital Buildings under jurisdiction of NHM Division Alwar (Annual Rate Contract)] [NIT NO. 05/2026-27(01)eemhalwar][2026_MEDIC_565647_1]</t>
+          <t>[Rate Contract for General Repair and Maintenance work at Various Hospital Buildings under jurisdiction of NHM Division Jaipur-I. (Civil, Sanitary, Joinery works)] [NIT 09 2026-27 divi jaipurI][2026_MEDIC_557384_1]</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1510,15 +1510,15 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>4,48,00,000</t>
+          <t>5,00,00,000</t>
         </is>
       </c>
       <c r="K19" t="n">
-        <v>44800000</v>
+        <v>50000000</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SslGsXAjXeu8uEKohFD43uQ%3D%3D</t>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SqdkfmioPRgMN%2BuVcWZkXJw%3D%3D</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Central eProcure</t>
+          <t>Rajasthan eProcurement</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1538,43 +1538,101 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2037.</t>
+          <t>5538.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>08-Jun-2026 04:00 PM</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>29-Jun-2026 06:00 PM</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>30-Jun-2026 01:00 PM</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>[Rate contract for General Repair and Maintenance Work at Various Hospital Buildings under jurisdiction of NHM Division Alwar (Annual Rate Contract)] [NIT NO. 05/2026-27(01)eemhalwar][2026_MEDIC_565647_1]</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Medical and Health||Chief Engineer</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>4,48,00,000</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>44800000</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://eproc.rajasthan.gov.in/nicgep/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=SslGsXAjXeu8uEKohFD43uQ%3D%3D</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Captured Backup</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Central eProcure</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2010.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>03-Jun-2026 06:00 PM</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>24-Jun-2026 06:00 PM</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>25-Jun-2026 06:05 PM</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>[Comprehensive Annual Repair Maintenance and Operations (ARMO) of ESIC Hospital and Staff Quarters at Kala Amb, Distt-Sirmour, HP- during 2026-27.] [W-17/1/2026/RO-PMD-Misc][2026_ESIC_911422_1]</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Employees State Insurance Corporation||R.O. Himachal Pradesh</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>1,30,03,957</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="K21" t="n">
         <v>13003957</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>https://eprocure.gov.in/eprocure/app?component=%24DirectLink&amp;page=FrontEndLatestActiveTenders&amp;service=direct&amp;session=T&amp;sp=Sc6oEKlA0tALrMKwrkHr0%2Fg%3D%3D</t>
         </is>

</xml_diff>